<commit_message>
chore(examples): update charts-line.xlsx demo file
</commit_message>
<xml_diff>
--- a/examples/excel/charts-line.xlsx
+++ b/examples/excel/charts-line.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -348,7 +348,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -834,7 +834,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:style val="3"/>
   <c:chart>
     <c:title>
@@ -1321,7 +1321,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -1809,7 +1809,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -2361,7 +2361,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -2720,7 +2720,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -2971,7 +2971,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart17.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -3130,7 +3130,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart18.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -3322,7 +3322,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart19.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -3823,7 +3823,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -3946,7 +3946,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart20.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -4458,7 +4458,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart21.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -4747,7 +4747,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart22.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -5112,7 +5112,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart23.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -5350,7 +5350,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart24.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -5687,7 +5687,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart25.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -5981,7 +5981,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart26.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -6191,7 +6191,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart27.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -6417,7 +6417,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart28.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -6904,7 +6904,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -7436,7 +7436,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -7597,7 +7597,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -8110,7 +8110,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -8407,7 +8407,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -8940,7 +8940,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:roundedCorners val="1"/>
   <c:chart>
     <c:title>
@@ -9459,7 +9459,7 @@
 </file>
 
 <file path=xl/drawings/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:chart>
     <c:title>
       <c:tx>
@@ -9972,7 +9972,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -10007,13 +10007,13 @@
     <xdr:from>
       <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -10035,15 +10035,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>37</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -10067,13 +10067,13 @@
     <xdr:from>
       <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>37</xdr:row>
+      <xdr:row>18</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -10097,7 +10097,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -10160,15 +10160,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>37</xdr:row>
+      <xdr:row>41</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -10222,7 +10222,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -10287,13 +10287,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>18</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>37</xdr:row>
+      <xdr:row>36</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -10347,7 +10347,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -10472,7 +10472,7 @@
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -10597,7 +10597,7 @@
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -10722,7 +10722,7 @@
 </file>
 
 <file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -11075,49 +11075,49 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
   <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re16f2ef06580438c"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
   <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R622d87bf24db424a"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
   <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R274a82bc11674dff"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
   <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb2c7f1920614886"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
   <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R727c62ff98bc43b9"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
   <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfee2e49219574a0b"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
   <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebf044d4fd7a4014"/>
 </x:worksheet>

</xml_diff>